<commit_message>
Fix VELA stock parsing: single colors, sizes in TALLA, SKU color codes
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/VELA_STOCK_COMPLETO.xlsx
+++ b/VELA_STOCK_COMPLETO.xlsx
@@ -1196,7 +1196,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Aguamarina/Negro</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G24" t="inlineStr"/>
@@ -1228,7 +1228,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Purpura/Negro</t>
+          <t>Purpura</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1260,7 +1260,7 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Azul Cielo/Blanco</t>
+          <t>Azul Cielo</t>
         </is>
       </c>
       <c r="G26" t="inlineStr"/>
@@ -1292,7 +1292,7 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Azul Marino/Rojo</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="G27" t="inlineStr"/>
@@ -1324,7 +1324,7 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Amarillo/Lila</t>
+          <t>Amarillo</t>
         </is>
       </c>
       <c r="G28" t="inlineStr"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3128,7 +3128,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3168,7 +3168,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3248,10 +3248,14 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr"/>
       <c r="H82" t="n">
         <v>7</v>
       </c>
@@ -3284,10 +3288,14 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr"/>
       <c r="H83" t="n">
         <v>10</v>
       </c>
@@ -3320,10 +3328,14 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr"/>
       <c r="H84" t="n">
         <v>5</v>
       </c>
@@ -3356,10 +3368,14 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
       <c r="H85" t="n">
         <v>2</v>
       </c>
@@ -3392,10 +3408,14 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr"/>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2XL</t>
+        </is>
+      </c>
       <c r="H86" t="n">
         <v>6</v>
       </c>
@@ -3428,10 +3448,14 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr"/>
       <c r="H87" t="n">
         <v>3</v>
       </c>
@@ -3464,10 +3488,14 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr"/>
       <c r="H88" t="n">
         <v>7</v>
       </c>
@@ -3500,10 +3528,14 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
       <c r="H89" t="n">
         <v>3</v>
       </c>
@@ -3536,10 +3568,14 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G90" t="inlineStr"/>
       <c r="H90" t="n">
         <v>6</v>
       </c>
@@ -3572,10 +3608,14 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr"/>
       <c r="H91" t="n">
         <v>2</v>
       </c>
@@ -4288,7 +4328,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -4564,7 +4604,7 @@
       <c r="E116" t="inlineStr"/>
       <c r="F116" t="inlineStr">
         <is>
-          <t>VERDE</t>
+          <t>Verde</t>
         </is>
       </c>
       <c r="G116" t="inlineStr"/>
@@ -4788,7 +4828,7 @@
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
@@ -9680,7 +9720,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -9720,7 +9760,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -9760,7 +9800,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -9960,7 +10000,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -10000,7 +10040,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -10040,7 +10080,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -10080,7 +10120,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -10120,7 +10160,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -10200,7 +10240,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -10240,7 +10280,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -10280,7 +10320,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -10480,7 +10520,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -10520,7 +10560,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
@@ -10560,7 +10600,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -10600,7 +10640,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -10640,7 +10680,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -10680,7 +10720,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -10720,7 +10760,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -10760,7 +10800,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
@@ -10800,7 +10840,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -10840,7 +10880,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
@@ -10880,7 +10920,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -10920,7 +10960,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -11160,7 +11200,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -11200,7 +11240,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -11240,7 +11280,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -11280,7 +11320,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -11320,7 +11360,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -11360,7 +11400,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -11400,7 +11440,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -11440,7 +11480,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -11480,7 +11520,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
@@ -11520,7 +11560,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
@@ -11560,7 +11600,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -11600,7 +11640,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -11640,7 +11680,7 @@
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
@@ -11680,7 +11720,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
@@ -13044,7 +13084,7 @@
       <c r="E337" t="inlineStr"/>
       <c r="F337" t="inlineStr">
         <is>
-          <t>CORAL</t>
+          <t>Coral</t>
         </is>
       </c>
       <c r="G337" t="inlineStr"/>
@@ -13076,7 +13116,7 @@
       <c r="E338" t="inlineStr"/>
       <c r="F338" t="inlineStr">
         <is>
-          <t>VERDE NEON</t>
+          <t>Verde Neon</t>
         </is>
       </c>
       <c r="G338" t="inlineStr"/>
@@ -13664,7 +13704,7 @@
       <c r="E356" t="inlineStr"/>
       <c r="F356" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G356" t="inlineStr"/>
@@ -13888,7 +13928,7 @@
       <c r="E363" t="inlineStr"/>
       <c r="F363" t="inlineStr">
         <is>
-          <t>MEDIANO</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="G363" t="inlineStr"/>
@@ -13920,7 +13960,7 @@
       <c r="E364" t="inlineStr"/>
       <c r="F364" t="inlineStr">
         <is>
-          <t>PEQUEÑO</t>
+          <t>Pequeño</t>
         </is>
       </c>
       <c r="G364" t="inlineStr"/>
@@ -13952,7 +13992,7 @@
       <c r="E365" t="inlineStr"/>
       <c r="F365" t="inlineStr">
         <is>
-          <t>GRANDE</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="G365" t="inlineStr"/>
@@ -14380,7 +14420,7 @@
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
@@ -14420,7 +14460,7 @@
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
@@ -14564,7 +14604,7 @@
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -14604,7 +14644,7 @@
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
@@ -15564,7 +15604,7 @@
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -15604,7 +15644,7 @@
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -15644,7 +15684,7 @@
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -15924,7 +15964,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -15964,7 +16004,7 @@
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -16004,7 +16044,7 @@
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -16140,7 +16180,7 @@
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
@@ -16212,7 +16252,7 @@
       <c r="E423" t="inlineStr"/>
       <c r="F423" t="inlineStr">
         <is>
-          <t>AZUL</t>
+          <t>Azul</t>
         </is>
       </c>
       <c r="G423" t="inlineStr"/>
@@ -21180,7 +21220,7 @@
       </c>
       <c r="F550" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G550" t="inlineStr">
@@ -21260,7 +21300,7 @@
       </c>
       <c r="F552" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G552" t="inlineStr">
@@ -21300,7 +21340,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G553" t="inlineStr">
@@ -21660,7 +21700,7 @@
       </c>
       <c r="F562" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G562" t="inlineStr">
@@ -22692,7 +22732,7 @@
       </c>
       <c r="F588" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G588" t="inlineStr">
@@ -22732,7 +22772,7 @@
       </c>
       <c r="F589" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G589" t="inlineStr">
@@ -22772,7 +22812,7 @@
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G590" t="inlineStr">
@@ -22812,7 +22852,7 @@
       </c>
       <c r="F591" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G591" t="inlineStr">
@@ -22852,7 +22892,7 @@
       </c>
       <c r="F592" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="G592" t="inlineStr">
@@ -23208,7 +23248,7 @@
       </c>
       <c r="F602" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G602" t="inlineStr">
@@ -23912,7 +23952,7 @@
       </c>
       <c r="F621" t="inlineStr">
         <is>
-          <t>PLAYUELA</t>
+          <t>Playuela</t>
         </is>
       </c>
       <c r="G621" t="inlineStr">
@@ -23952,7 +23992,7 @@
       </c>
       <c r="F622" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="G622" t="inlineStr">
@@ -23992,7 +24032,7 @@
       </c>
       <c r="F623" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="G623" t="inlineStr">
@@ -24704,7 +24744,7 @@
       </c>
       <c r="F641" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G641" t="inlineStr">
@@ -25040,7 +25080,7 @@
       </c>
       <c r="F650" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G650" t="inlineStr">
@@ -25080,7 +25120,7 @@
       </c>
       <c r="F651" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G651" t="inlineStr">
@@ -25548,10 +25588,14 @@
       <c r="E663" t="inlineStr"/>
       <c r="F663" t="inlineStr">
         <is>
-          <t>Negro, P</t>
-        </is>
-      </c>
-      <c r="G663" t="inlineStr"/>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="H663" t="n">
         <v>1</v>
       </c>
@@ -25580,10 +25624,14 @@
       <c r="E664" t="inlineStr"/>
       <c r="F664" t="inlineStr">
         <is>
-          <t>Blanco, P</t>
-        </is>
-      </c>
-      <c r="G664" t="inlineStr"/>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="H664" t="n">
         <v>13</v>
       </c>
@@ -26856,7 +26904,7 @@
       </c>
       <c r="F696" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G696" t="inlineStr">
@@ -26896,7 +26944,7 @@
       </c>
       <c r="F697" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G697" t="inlineStr">
@@ -26936,7 +26984,7 @@
       </c>
       <c r="F698" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G698" t="inlineStr">
@@ -26976,7 +27024,7 @@
       </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G699" t="inlineStr">
@@ -27016,7 +27064,7 @@
       </c>
       <c r="F700" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="G700" t="inlineStr">
@@ -27376,7 +27424,7 @@
       </c>
       <c r="F709" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G709" t="inlineStr">
@@ -27416,7 +27464,7 @@
       </c>
       <c r="F710" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G710" t="inlineStr">
@@ -27456,7 +27504,7 @@
       </c>
       <c r="F711" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G711" t="inlineStr">
@@ -27496,7 +27544,7 @@
       </c>
       <c r="F712" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G712" t="inlineStr">
@@ -27576,7 +27624,7 @@
       </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G714" t="inlineStr">
@@ -27616,7 +27664,7 @@
       </c>
       <c r="F715" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G715" t="inlineStr">
@@ -28128,7 +28176,7 @@
       </c>
       <c r="F728" t="inlineStr">
         <is>
-          <t>FRAILE</t>
+          <t>Fraile</t>
         </is>
       </c>
       <c r="G728" t="inlineStr">
@@ -29948,10 +29996,14 @@
       <c r="E776" t="inlineStr"/>
       <c r="F776" t="inlineStr">
         <is>
-          <t>Verde Militar, P</t>
-        </is>
-      </c>
-      <c r="G776" t="inlineStr"/>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="H776" t="n">
         <v>2</v>
       </c>
@@ -30188,7 +30240,7 @@
       <c r="E783" t="inlineStr"/>
       <c r="F783" t="inlineStr">
         <is>
-          <t>Ondas/Verde</t>
+          <t>Ondas</t>
         </is>
       </c>
       <c r="G783" t="inlineStr"/>
@@ -30220,7 +30272,7 @@
       <c r="E784" t="inlineStr"/>
       <c r="F784" t="inlineStr">
         <is>
-          <t>Ovalo/Azul</t>
+          <t>Ovalo</t>
         </is>
       </c>
       <c r="G784" t="inlineStr"/>
@@ -30252,7 +30304,7 @@
       <c r="E785" t="inlineStr"/>
       <c r="F785" t="inlineStr">
         <is>
-          <t>Daily/Negro</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="G785" t="inlineStr"/>
@@ -30408,7 +30460,7 @@
       </c>
       <c r="F789" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G789" t="inlineStr">
@@ -33680,7 +33732,7 @@
       </c>
       <c r="F877" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G877" t="inlineStr">
@@ -33720,7 +33772,7 @@
       </c>
       <c r="F878" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G878" t="inlineStr">
@@ -33840,7 +33892,7 @@
       </c>
       <c r="F881" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G881" t="inlineStr">
@@ -33880,7 +33932,7 @@
       </c>
       <c r="F882" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G882" t="inlineStr">
@@ -33920,7 +33972,7 @@
       </c>
       <c r="F883" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G883" t="inlineStr">
@@ -33960,7 +34012,7 @@
       </c>
       <c r="F884" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G884" t="inlineStr">
@@ -34000,7 +34052,7 @@
       </c>
       <c r="F885" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G885" t="inlineStr">
@@ -34040,7 +34092,7 @@
       </c>
       <c r="F886" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G886" t="inlineStr">
@@ -34080,7 +34132,7 @@
       </c>
       <c r="F887" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G887" t="inlineStr">
@@ -34120,7 +34172,7 @@
       </c>
       <c r="F888" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G888" t="inlineStr">
@@ -34160,7 +34212,7 @@
       </c>
       <c r="F889" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G889" t="inlineStr">
@@ -34200,7 +34252,7 @@
       </c>
       <c r="F890" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G890" t="inlineStr">
@@ -41560,7 +41612,7 @@
       </c>
       <c r="F1074" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1074" t="inlineStr">
@@ -42280,7 +42332,7 @@
       </c>
       <c r="F1092" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1092" t="inlineStr">
@@ -42320,7 +42372,7 @@
       </c>
       <c r="F1093" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1093" t="inlineStr">
@@ -42360,7 +42412,7 @@
       </c>
       <c r="F1094" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1094" t="inlineStr">
@@ -42480,7 +42532,7 @@
       </c>
       <c r="F1097" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G1097" t="inlineStr">
@@ -42520,7 +42572,7 @@
       </c>
       <c r="F1098" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1098" t="inlineStr">
@@ -42560,7 +42612,7 @@
       </c>
       <c r="F1099" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1099" t="inlineStr">
@@ -42596,7 +42648,7 @@
       <c r="E1100" t="inlineStr"/>
       <c r="F1100" t="inlineStr">
         <is>
-          <t>VERDE NEON</t>
+          <t>Verde Neon</t>
         </is>
       </c>
       <c r="G1100" t="inlineStr"/>
@@ -43112,7 +43164,7 @@
       </c>
       <c r="F1115" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1115" t="inlineStr">
@@ -43152,7 +43204,7 @@
       </c>
       <c r="F1116" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1116" t="inlineStr">
@@ -43192,7 +43244,7 @@
       </c>
       <c r="F1117" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1117" t="inlineStr">
@@ -43232,7 +43284,7 @@
       </c>
       <c r="F1118" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1118" t="inlineStr">
@@ -43272,7 +43324,7 @@
       </c>
       <c r="F1119" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1119" t="inlineStr">
@@ -43312,7 +43364,7 @@
       </c>
       <c r="F1120" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1120" t="inlineStr">
@@ -43352,7 +43404,7 @@
       </c>
       <c r="F1121" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1121" t="inlineStr">
@@ -43392,7 +43444,7 @@
       </c>
       <c r="F1122" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1122" t="inlineStr">
@@ -43432,7 +43484,7 @@
       </c>
       <c r="F1123" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1123" t="inlineStr">
@@ -47392,7 +47444,7 @@
       </c>
       <c r="F1222" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1222" t="inlineStr">
@@ -47432,7 +47484,7 @@
       </c>
       <c r="F1223" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1223" t="inlineStr">
@@ -47712,7 +47764,7 @@
       </c>
       <c r="F1230" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="G1230" t="inlineStr">
@@ -47752,7 +47804,7 @@
       </c>
       <c r="F1231" t="inlineStr">
         <is>
-          <t>PLAYUELA</t>
+          <t>Playuela</t>
         </is>
       </c>
       <c r="G1231" t="inlineStr">
@@ -47792,7 +47844,7 @@
       </c>
       <c r="F1232" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1232" t="inlineStr">
@@ -47832,7 +47884,7 @@
       </c>
       <c r="F1233" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1233" t="inlineStr">
@@ -47872,7 +47924,7 @@
       </c>
       <c r="F1234" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1234" t="inlineStr">
@@ -47912,7 +47964,7 @@
       </c>
       <c r="F1235" t="inlineStr">
         <is>
-          <t>PLAYUELA</t>
+          <t>Playuela</t>
         </is>
       </c>
       <c r="G1235" t="inlineStr">
@@ -47952,7 +48004,7 @@
       </c>
       <c r="F1236" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="G1236" t="inlineStr">
@@ -48032,7 +48084,7 @@
       </c>
       <c r="F1238" t="inlineStr">
         <is>
-          <t>TUCUPIDO</t>
+          <t>Tucupido</t>
         </is>
       </c>
       <c r="G1238" t="inlineStr">
@@ -48072,7 +48124,7 @@
       </c>
       <c r="F1239" t="inlineStr">
         <is>
-          <t>PLAYUELA</t>
+          <t>Playuela</t>
         </is>
       </c>
       <c r="G1239" t="inlineStr">
@@ -48112,7 +48164,7 @@
       </c>
       <c r="F1240" t="inlineStr">
         <is>
-          <t>SOMBRERO</t>
+          <t>Sombrero</t>
         </is>
       </c>
       <c r="G1240" t="inlineStr">
@@ -48152,7 +48204,7 @@
       </c>
       <c r="F1241" t="inlineStr">
         <is>
-          <t>SAL</t>
+          <t>Sal</t>
         </is>
       </c>
       <c r="G1241" t="inlineStr">
@@ -50624,7 +50676,7 @@
       </c>
       <c r="F1304" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1304" t="inlineStr">
@@ -50664,7 +50716,7 @@
       </c>
       <c r="F1305" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1305" t="inlineStr">
@@ -50784,7 +50836,7 @@
       </c>
       <c r="F1308" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1308" t="inlineStr">
@@ -50944,7 +50996,7 @@
       </c>
       <c r="F1312" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1312" t="inlineStr">
@@ -51064,7 +51116,7 @@
       </c>
       <c r="F1315" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1315" t="inlineStr">
@@ -51104,7 +51156,7 @@
       </c>
       <c r="F1316" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1316" t="inlineStr">
@@ -51144,7 +51196,7 @@
       </c>
       <c r="F1317" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1317" t="inlineStr">
@@ -51184,7 +51236,7 @@
       </c>
       <c r="F1318" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1318" t="inlineStr">
@@ -51224,7 +51276,7 @@
       </c>
       <c r="F1319" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1319" t="inlineStr">
@@ -51264,7 +51316,7 @@
       </c>
       <c r="F1320" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1320" t="inlineStr">
@@ -51304,7 +51356,7 @@
       </c>
       <c r="F1321" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1321" t="inlineStr">
@@ -51344,7 +51396,7 @@
       </c>
       <c r="F1322" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1322" t="inlineStr">
@@ -54406,13 +54458,13 @@
       </c>
       <c r="D1401" t="inlineStr">
         <is>
-          <t>CUADRO BAND VENEZUELA</t>
+          <t>CUADRO BAND</t>
         </is>
       </c>
       <c r="E1401" t="inlineStr"/>
       <c r="F1401" t="inlineStr">
         <is>
-          <t>BAND VENEZUELA</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="G1401" t="inlineStr"/>
@@ -55640,7 +55692,7 @@
       <c r="E1434" t="inlineStr"/>
       <c r="F1434" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1434" t="inlineStr"/>
@@ -56256,7 +56308,7 @@
       <c r="E1453" t="inlineStr"/>
       <c r="F1453" t="inlineStr">
         <is>
-          <t>Azul Marino/Rojo</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="G1453" t="inlineStr"/>
@@ -57124,10 +57176,14 @@
       </c>
       <c r="F1480" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1480" t="inlineStr">
+        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G1480" t="inlineStr"/>
       <c r="H1480" t="n">
         <v>1</v>
       </c>
@@ -57160,10 +57216,14 @@
       </c>
       <c r="F1481" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1481" t="inlineStr">
+        <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="G1481" t="inlineStr"/>
       <c r="H1481" t="n">
         <v>2</v>
       </c>
@@ -57196,10 +57256,14 @@
       </c>
       <c r="F1482" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1482" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G1482" t="inlineStr"/>
       <c r="H1482" t="n">
         <v>4</v>
       </c>
@@ -57232,10 +57296,14 @@
       </c>
       <c r="F1483" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1483" t="inlineStr">
+        <is>
           <t>M</t>
         </is>
       </c>
-      <c r="G1483" t="inlineStr"/>
       <c r="H1483" t="n">
         <v>2</v>
       </c>
@@ -57268,10 +57336,14 @@
       </c>
       <c r="F1484" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1484" t="inlineStr">
+        <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="G1484" t="inlineStr"/>
       <c r="H1484" t="n">
         <v>3</v>
       </c>
@@ -57304,7 +57376,7 @@
       </c>
       <c r="F1485" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1485" t="inlineStr">
@@ -57344,7 +57416,7 @@
       </c>
       <c r="F1486" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1486" t="inlineStr">
@@ -57384,10 +57456,14 @@
       </c>
       <c r="F1487" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1487" t="inlineStr">
+        <is>
           <t>L</t>
         </is>
       </c>
-      <c r="G1487" t="inlineStr"/>
       <c r="H1487" t="n">
         <v>3</v>
       </c>
@@ -57420,10 +57496,14 @@
       </c>
       <c r="F1488" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1488" t="inlineStr">
+        <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="G1488" t="inlineStr"/>
       <c r="H1488" t="n">
         <v>3</v>
       </c>
@@ -57456,7 +57536,7 @@
       </c>
       <c r="F1489" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1489" t="inlineStr">
@@ -57496,10 +57576,14 @@
       </c>
       <c r="F1490" t="inlineStr">
         <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="G1490" t="inlineStr"/>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1490" t="inlineStr">
+        <is>
+          <t>2XL</t>
+        </is>
+      </c>
       <c r="H1490" t="n">
         <v>3</v>
       </c>
@@ -58936,7 +59020,7 @@
       </c>
       <c r="F1527" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1527" t="inlineStr">
@@ -58976,7 +59060,7 @@
       </c>
       <c r="F1528" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1528" t="inlineStr">
@@ -59016,7 +59100,7 @@
       </c>
       <c r="F1529" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1529" t="inlineStr">
@@ -59056,7 +59140,7 @@
       </c>
       <c r="F1530" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1530" t="inlineStr">
@@ -59216,7 +59300,7 @@
       </c>
       <c r="F1534" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1534" t="inlineStr">
@@ -59256,7 +59340,7 @@
       </c>
       <c r="F1535" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1535" t="inlineStr">
@@ -59296,7 +59380,7 @@
       </c>
       <c r="F1536" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1536" t="inlineStr">
@@ -59452,7 +59536,7 @@
       <c r="E1540" t="inlineStr"/>
       <c r="F1540" t="inlineStr">
         <is>
-          <t>Made in Venezuela/Verde</t>
+          <t>Made in Venezuela</t>
         </is>
       </c>
       <c r="G1540" t="inlineStr"/>
@@ -59484,7 +59568,7 @@
       <c r="E1541" t="inlineStr"/>
       <c r="F1541" t="inlineStr">
         <is>
-          <t>Ovalo/Azul</t>
+          <t>Ovalo</t>
         </is>
       </c>
       <c r="G1541" t="inlineStr"/>
@@ -59516,7 +59600,7 @@
       <c r="E1542" t="inlineStr"/>
       <c r="F1542" t="inlineStr">
         <is>
-          <t>Daily/Negro</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="G1542" t="inlineStr"/>
@@ -61148,7 +61232,7 @@
       <c r="E1584" t="inlineStr"/>
       <c r="F1584" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1584" t="inlineStr"/>
@@ -61184,7 +61268,7 @@
       </c>
       <c r="F1585" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1585" t="inlineStr">
@@ -61224,7 +61308,7 @@
       </c>
       <c r="F1586" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1586" t="inlineStr">
@@ -61368,7 +61452,7 @@
       </c>
       <c r="F1590" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1590" t="inlineStr">
@@ -61408,7 +61492,7 @@
       </c>
       <c r="F1591" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1591" t="inlineStr">
@@ -61768,7 +61852,7 @@
       <c r="E1601" t="inlineStr"/>
       <c r="F1601" t="inlineStr">
         <is>
-          <t>GRANDE</t>
+          <t>Grande</t>
         </is>
       </c>
       <c r="G1601" t="inlineStr"/>
@@ -62160,7 +62244,7 @@
       <c r="E1612" t="inlineStr"/>
       <c r="F1612" t="inlineStr">
         <is>
-          <t>Azul Cielo/Blanco</t>
+          <t>Azul Cielo</t>
         </is>
       </c>
       <c r="G1612" t="inlineStr"/>
@@ -62304,7 +62388,7 @@
       <c r="E1616" t="inlineStr"/>
       <c r="F1616" t="inlineStr">
         <is>
-          <t>Amarillo/Lila</t>
+          <t>Amarillo</t>
         </is>
       </c>
       <c r="G1616" t="inlineStr"/>
@@ -62908,7 +62992,7 @@
       </c>
       <c r="F1633" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1633" t="inlineStr">
@@ -62944,7 +63028,7 @@
       <c r="E1634" t="inlineStr"/>
       <c r="F1634" t="inlineStr">
         <is>
-          <t>Aguamarina/Negro</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1634" t="inlineStr"/>
@@ -62976,7 +63060,7 @@
       <c r="E1635" t="inlineStr"/>
       <c r="F1635" t="inlineStr">
         <is>
-          <t>Purpura/Negro</t>
+          <t>Purpura</t>
         </is>
       </c>
       <c r="G1635" t="inlineStr"/>
@@ -63076,7 +63160,7 @@
       </c>
       <c r="F1638" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1638" t="inlineStr">
@@ -63284,7 +63368,7 @@
       </c>
       <c r="F1644" t="inlineStr">
         <is>
-          <t>AGUAMARINA</t>
+          <t>Aguamarina</t>
         </is>
       </c>
       <c r="G1644" t="inlineStr">
@@ -63364,7 +63448,7 @@
       </c>
       <c r="F1646" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1646" t="inlineStr">
@@ -64968,7 +65052,7 @@
       </c>
       <c r="F1687" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1687" t="inlineStr">
@@ -65840,7 +65924,7 @@
       </c>
       <c r="F1710" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1710" t="inlineStr">
@@ -65876,7 +65960,7 @@
       <c r="E1711" t="inlineStr"/>
       <c r="F1711" t="inlineStr">
         <is>
-          <t>VERDE</t>
+          <t>Verde</t>
         </is>
       </c>
       <c r="G1711" t="inlineStr"/>
@@ -66144,7 +66228,7 @@
       </c>
       <c r="F1718" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G1718" t="inlineStr">
@@ -66556,7 +66640,7 @@
       </c>
       <c r="F1729" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G1729" t="inlineStr">
@@ -66596,7 +66680,7 @@
       </c>
       <c r="F1730" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1730" t="inlineStr">
@@ -66636,7 +66720,7 @@
       </c>
       <c r="F1731" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1731" t="inlineStr">
@@ -66796,7 +66880,7 @@
       </c>
       <c r="F1735" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1735" t="inlineStr">
@@ -67116,7 +67200,7 @@
       </c>
       <c r="F1743" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1743" t="inlineStr">
@@ -67178,12 +67262,24 @@
       </c>
       <c r="D1745" t="inlineStr">
         <is>
-          <t>PANNKI33T2</t>
-        </is>
-      </c>
-      <c r="E1745" t="inlineStr"/>
-      <c r="F1745" t="inlineStr"/>
-      <c r="G1745" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1745" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1745" t="inlineStr">
+        <is>
+          <t>Kaki</t>
+        </is>
+      </c>
+      <c r="G1745" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="H1745" t="n">
         <v>2</v>
       </c>
@@ -67206,12 +67302,24 @@
       </c>
       <c r="D1746" t="inlineStr">
         <is>
-          <t>PANNKI33T4</t>
-        </is>
-      </c>
-      <c r="E1746" t="inlineStr"/>
-      <c r="F1746" t="inlineStr"/>
-      <c r="G1746" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1746" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1746" t="inlineStr">
+        <is>
+          <t>Kaki</t>
+        </is>
+      </c>
+      <c r="G1746" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H1746" t="n">
         <v>2</v>
       </c>
@@ -67234,12 +67342,24 @@
       </c>
       <c r="D1747" t="inlineStr">
         <is>
-          <t>PANNKI33T6</t>
-        </is>
-      </c>
-      <c r="E1747" t="inlineStr"/>
-      <c r="F1747" t="inlineStr"/>
-      <c r="G1747" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1747" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1747" t="inlineStr">
+        <is>
+          <t>Kaki</t>
+        </is>
+      </c>
+      <c r="G1747" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="H1747" t="n">
         <v>2</v>
       </c>
@@ -67262,12 +67382,24 @@
       </c>
       <c r="D1748" t="inlineStr">
         <is>
-          <t>PANNKI33T12</t>
-        </is>
-      </c>
-      <c r="E1748" t="inlineStr"/>
-      <c r="F1748" t="inlineStr"/>
-      <c r="G1748" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1748" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1748" t="inlineStr">
+        <is>
+          <t>Kaki</t>
+        </is>
+      </c>
+      <c r="G1748" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="H1748" t="n">
         <v>2</v>
       </c>
@@ -67290,12 +67422,24 @@
       </c>
       <c r="D1749" t="inlineStr">
         <is>
-          <t>PANNKI12T2</t>
-        </is>
-      </c>
-      <c r="E1749" t="inlineStr"/>
-      <c r="F1749" t="inlineStr"/>
-      <c r="G1749" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1749" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1749" t="inlineStr">
+        <is>
+          <t>Azul Marino</t>
+        </is>
+      </c>
+      <c r="G1749" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="H1749" t="n">
         <v>1</v>
       </c>
@@ -67318,12 +67462,24 @@
       </c>
       <c r="D1750" t="inlineStr">
         <is>
-          <t>PANNKI12T4</t>
-        </is>
-      </c>
-      <c r="E1750" t="inlineStr"/>
-      <c r="F1750" t="inlineStr"/>
-      <c r="G1750" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1750" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1750" t="inlineStr">
+        <is>
+          <t>Azul Marino</t>
+        </is>
+      </c>
+      <c r="G1750" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H1750" t="n">
         <v>3</v>
       </c>
@@ -67346,12 +67502,24 @@
       </c>
       <c r="D1751" t="inlineStr">
         <is>
-          <t>PANNKI12T6</t>
-        </is>
-      </c>
-      <c r="E1751" t="inlineStr"/>
-      <c r="F1751" t="inlineStr"/>
-      <c r="G1751" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1751" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1751" t="inlineStr">
+        <is>
+          <t>Azul Marino</t>
+        </is>
+      </c>
+      <c r="G1751" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="H1751" t="n">
         <v>1</v>
       </c>
@@ -67374,12 +67542,24 @@
       </c>
       <c r="D1752" t="inlineStr">
         <is>
-          <t>PANNKI12T8</t>
-        </is>
-      </c>
-      <c r="E1752" t="inlineStr"/>
-      <c r="F1752" t="inlineStr"/>
-      <c r="G1752" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1752" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1752" t="inlineStr">
+        <is>
+          <t>Azul Marino</t>
+        </is>
+      </c>
+      <c r="G1752" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="H1752" t="n">
         <v>1</v>
       </c>
@@ -67402,12 +67582,24 @@
       </c>
       <c r="D1753" t="inlineStr">
         <is>
-          <t>PANNKI12T10</t>
-        </is>
-      </c>
-      <c r="E1753" t="inlineStr"/>
-      <c r="F1753" t="inlineStr"/>
-      <c r="G1753" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1753" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1753" t="inlineStr">
+        <is>
+          <t>Azul Marino</t>
+        </is>
+      </c>
+      <c r="G1753" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H1753" t="n">
         <v>1</v>
       </c>
@@ -67430,12 +67622,24 @@
       </c>
       <c r="D1754" t="inlineStr">
         <is>
-          <t>PANNKI12T12</t>
-        </is>
-      </c>
-      <c r="E1754" t="inlineStr"/>
-      <c r="F1754" t="inlineStr"/>
-      <c r="G1754" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1754" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1754" t="inlineStr">
+        <is>
+          <t>Azul Marino</t>
+        </is>
+      </c>
+      <c r="G1754" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="H1754" t="n">
         <v>1</v>
       </c>
@@ -67458,12 +67662,24 @@
       </c>
       <c r="D1755" t="inlineStr">
         <is>
-          <t>PANNKI43T2</t>
-        </is>
-      </c>
-      <c r="E1755" t="inlineStr"/>
-      <c r="F1755" t="inlineStr"/>
-      <c r="G1755" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1755" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1755" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G1755" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="H1755" t="n">
         <v>2</v>
       </c>
@@ -67486,12 +67702,24 @@
       </c>
       <c r="D1756" t="inlineStr">
         <is>
-          <t>PANNKI43T4</t>
-        </is>
-      </c>
-      <c r="E1756" t="inlineStr"/>
-      <c r="F1756" t="inlineStr"/>
-      <c r="G1756" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1756" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1756" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G1756" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H1756" t="n">
         <v>2</v>
       </c>
@@ -67514,12 +67742,24 @@
       </c>
       <c r="D1757" t="inlineStr">
         <is>
-          <t>PANNKI43T6</t>
-        </is>
-      </c>
-      <c r="E1757" t="inlineStr"/>
-      <c r="F1757" t="inlineStr"/>
-      <c r="G1757" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1757" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1757" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G1757" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="H1757" t="n">
         <v>2</v>
       </c>
@@ -67542,12 +67782,24 @@
       </c>
       <c r="D1758" t="inlineStr">
         <is>
-          <t>PANNKI43T8</t>
-        </is>
-      </c>
-      <c r="E1758" t="inlineStr"/>
-      <c r="F1758" t="inlineStr"/>
-      <c r="G1758" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1758" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1758" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G1758" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="H1758" t="n">
         <v>2</v>
       </c>
@@ -67570,12 +67822,24 @@
       </c>
       <c r="D1759" t="inlineStr">
         <is>
-          <t>PANNKI43T10</t>
-        </is>
-      </c>
-      <c r="E1759" t="inlineStr"/>
-      <c r="F1759" t="inlineStr"/>
-      <c r="G1759" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1759" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1759" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G1759" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H1759" t="n">
         <v>2</v>
       </c>
@@ -67598,12 +67862,24 @@
       </c>
       <c r="D1760" t="inlineStr">
         <is>
-          <t>PANNKI43T12</t>
-        </is>
-      </c>
-      <c r="E1760" t="inlineStr"/>
-      <c r="F1760" t="inlineStr"/>
-      <c r="G1760" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1760" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1760" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="G1760" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="H1760" t="n">
         <v>4</v>
       </c>
@@ -67626,12 +67902,24 @@
       </c>
       <c r="D1761" t="inlineStr">
         <is>
-          <t>PANNKI66T2</t>
-        </is>
-      </c>
-      <c r="E1761" t="inlineStr"/>
-      <c r="F1761" t="inlineStr"/>
-      <c r="G1761" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1761" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1761" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G1761" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="H1761" t="n">
         <v>2</v>
       </c>
@@ -67654,12 +67942,24 @@
       </c>
       <c r="D1762" t="inlineStr">
         <is>
-          <t>PANNKI66T4</t>
-        </is>
-      </c>
-      <c r="E1762" t="inlineStr"/>
-      <c r="F1762" t="inlineStr"/>
-      <c r="G1762" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1762" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1762" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G1762" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H1762" t="n">
         <v>2</v>
       </c>
@@ -67682,12 +67982,24 @@
       </c>
       <c r="D1763" t="inlineStr">
         <is>
-          <t>PANNKI66T6</t>
-        </is>
-      </c>
-      <c r="E1763" t="inlineStr"/>
-      <c r="F1763" t="inlineStr"/>
-      <c r="G1763" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1763" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1763" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G1763" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="H1763" t="n">
         <v>2</v>
       </c>
@@ -67710,12 +68022,24 @@
       </c>
       <c r="D1764" t="inlineStr">
         <is>
-          <t>PANNKI66T8</t>
-        </is>
-      </c>
-      <c r="E1764" t="inlineStr"/>
-      <c r="F1764" t="inlineStr"/>
-      <c r="G1764" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1764" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1764" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G1764" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="H1764" t="n">
         <v>2</v>
       </c>
@@ -67738,12 +68062,24 @@
       </c>
       <c r="D1765" t="inlineStr">
         <is>
-          <t>PANNKI66T10</t>
-        </is>
-      </c>
-      <c r="E1765" t="inlineStr"/>
-      <c r="F1765" t="inlineStr"/>
-      <c r="G1765" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1765" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1765" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G1765" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="H1765" t="n">
         <v>3</v>
       </c>
@@ -67766,12 +68102,24 @@
       </c>
       <c r="D1766" t="inlineStr">
         <is>
-          <t>PANNKI66T12</t>
-        </is>
-      </c>
-      <c r="E1766" t="inlineStr"/>
-      <c r="F1766" t="inlineStr"/>
-      <c r="G1766" t="inlineStr"/>
+          <t>PANNKI</t>
+        </is>
+      </c>
+      <c r="E1766" t="inlineStr">
+        <is>
+          <t>KIDS</t>
+        </is>
+      </c>
+      <c r="F1766" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G1766" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="H1766" t="n">
         <v>2</v>
       </c>
@@ -69716,7 +70064,7 @@
       </c>
       <c r="F1815" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1815" t="inlineStr">
@@ -69756,7 +70104,7 @@
       </c>
       <c r="F1816" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1816" t="inlineStr">
@@ -69980,7 +70328,7 @@
       </c>
       <c r="F1822" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1822" t="inlineStr">
@@ -70156,7 +70504,7 @@
       </c>
       <c r="F1827" t="inlineStr">
         <is>
-          <t>FRAILE</t>
+          <t>Fraile</t>
         </is>
       </c>
       <c r="G1827" t="inlineStr">
@@ -70196,7 +70544,7 @@
       </c>
       <c r="F1828" t="inlineStr">
         <is>
-          <t>CRASQUI</t>
+          <t>Crasqui</t>
         </is>
       </c>
       <c r="G1828" t="inlineStr">
@@ -70236,7 +70584,7 @@
       </c>
       <c r="F1829" t="inlineStr">
         <is>
-          <t>ROYAL</t>
+          <t>Royal</t>
         </is>
       </c>
       <c r="G1829" t="inlineStr">
@@ -70276,7 +70624,7 @@
       </c>
       <c r="F1830" t="inlineStr">
         <is>
-          <t>BLACK ABSTRACT</t>
+          <t>Black Abstract</t>
         </is>
       </c>
       <c r="G1830" t="inlineStr">
@@ -70316,7 +70664,7 @@
       </c>
       <c r="F1831" t="inlineStr">
         <is>
-          <t>DORADO</t>
+          <t>Dorado</t>
         </is>
       </c>
       <c r="G1831" t="inlineStr">
@@ -70356,7 +70704,7 @@
       </c>
       <c r="F1832" t="inlineStr">
         <is>
-          <t>CRASQUI</t>
+          <t>Crasqui</t>
         </is>
       </c>
       <c r="G1832" t="inlineStr">
@@ -70396,7 +70744,7 @@
       </c>
       <c r="F1833" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1833" t="inlineStr">
@@ -70436,10 +70784,14 @@
       </c>
       <c r="F1834" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1834" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G1834" t="inlineStr"/>
       <c r="H1834" t="n">
         <v>1</v>
       </c>
@@ -70664,7 +71016,7 @@
       </c>
       <c r="F1840" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G1840" t="inlineStr">
@@ -70864,7 +71216,7 @@
       </c>
       <c r="F1845" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1845" t="inlineStr">
@@ -71124,10 +71476,14 @@
       <c r="E1853" t="inlineStr"/>
       <c r="F1853" t="inlineStr">
         <is>
-          <t>Azul Lavanda, P</t>
-        </is>
-      </c>
-      <c r="G1853" t="inlineStr"/>
+          <t>Azul Lavanda</t>
+        </is>
+      </c>
+      <c r="G1853" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="H1853" t="n">
         <v>3</v>
       </c>
@@ -71156,10 +71512,14 @@
       <c r="E1854" t="inlineStr"/>
       <c r="F1854" t="inlineStr">
         <is>
-          <t>Verde Militar, P</t>
-        </is>
-      </c>
-      <c r="G1854" t="inlineStr"/>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="G1854" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="H1854" t="n">
         <v>3</v>
       </c>
@@ -71260,10 +71620,14 @@
       <c r="E1857" t="inlineStr"/>
       <c r="F1857" t="inlineStr">
         <is>
-          <t>Blanco, P</t>
-        </is>
-      </c>
-      <c r="G1857" t="inlineStr"/>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1857" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
       <c r="H1857" t="n">
         <v>3</v>
       </c>
@@ -71376,7 +71740,7 @@
       </c>
       <c r="F1860" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1860" t="inlineStr">
@@ -71456,7 +71820,7 @@
       </c>
       <c r="F1862" t="inlineStr">
         <is>
-          <t>Blanco/ Nueva Esparta</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1862" t="inlineStr">
@@ -72052,7 +72416,7 @@
       <c r="E1878" t="inlineStr"/>
       <c r="F1878" t="inlineStr">
         <is>
-          <t>CORAL</t>
+          <t>Coral</t>
         </is>
       </c>
       <c r="G1878" t="inlineStr"/>
@@ -73316,7 +73680,7 @@
       <c r="E1910" t="inlineStr"/>
       <c r="F1910" t="inlineStr">
         <is>
-          <t>Palmeras/Azul</t>
+          <t>Palmeras</t>
         </is>
       </c>
       <c r="G1910" t="inlineStr"/>
@@ -73348,7 +73712,7 @@
       <c r="E1911" t="inlineStr"/>
       <c r="F1911" t="inlineStr">
         <is>
-          <t>PEQUEÑO</t>
+          <t>Pequeño</t>
         </is>
       </c>
       <c r="G1911" t="inlineStr"/>
@@ -73424,7 +73788,7 @@
       </c>
       <c r="F1913" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1913" t="inlineStr">
@@ -73464,7 +73828,7 @@
       </c>
       <c r="F1914" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1914" t="inlineStr">
@@ -73580,7 +73944,7 @@
       <c r="E1917" t="inlineStr"/>
       <c r="F1917" t="inlineStr">
         <is>
-          <t>AZUL</t>
+          <t>Azul</t>
         </is>
       </c>
       <c r="G1917" t="inlineStr"/>
@@ -74128,7 +74492,7 @@
       </c>
       <c r="F1931" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1931" t="inlineStr">
@@ -74320,7 +74684,7 @@
       </c>
       <c r="F1936" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G1936" t="inlineStr">
@@ -74360,7 +74724,7 @@
       </c>
       <c r="F1937" t="inlineStr">
         <is>
-          <t>BLANCO</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="G1937" t="inlineStr">
@@ -74512,7 +74876,7 @@
       <c r="E1941" t="inlineStr"/>
       <c r="F1941" t="inlineStr">
         <is>
-          <t>MEDIANO</t>
+          <t>Mediano</t>
         </is>
       </c>
       <c r="G1941" t="inlineStr"/>
@@ -74588,7 +74952,7 @@
       </c>
       <c r="F1943" t="inlineStr">
         <is>
-          <t>NEGRO</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="G1943" t="inlineStr">
@@ -74668,7 +75032,7 @@
       </c>
       <c r="F1945" t="inlineStr">
         <is>
-          <t>VERDE MILITAR</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="G1945" t="inlineStr">
@@ -74980,10 +75344,14 @@
       </c>
       <c r="F1953" t="inlineStr">
         <is>
+          <t>Blanco</t>
+        </is>
+      </c>
+      <c r="G1953" t="inlineStr">
+        <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G1953" t="inlineStr"/>
       <c r="H1953" t="n">
         <v>1</v>
       </c>

</xml_diff>